<commit_message>
Restore Byxelkrok in station code list
The Byxelkrok row (BYXE, 00103946) was accidentally overwritten
when the plain Ängskärsklubb row was added in d7c0ef6.
</commit_message>
<xml_diff>
--- a/inst/extdata/codelist.xlsx
+++ b/inst/extdata/codelist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\annesore\github\MoCiS2\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{524D8DB3-AF48-4CA1-B9C2-E8D3572652F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8329D15B-2FC4-483C-8994-189B0AEA2B1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2250" yWindow="450" windowWidth="19950" windowHeight="20115" tabRatio="877" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1755" uniqueCount="729">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1759" uniqueCount="732">
   <si>
     <t>PERC</t>
   </si>
@@ -2223,6 +2223,15 @@
   </si>
   <si>
     <t>CH07/895</t>
+  </si>
+  <si>
+    <t>BYXE</t>
+  </si>
+  <si>
+    <t>00103946</t>
+  </si>
+  <si>
+    <t>Byxelkrok</t>
   </si>
 </sst>
 </file>
@@ -2717,7 +2726,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D95"/>
+  <dimension ref="A1:D96"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="25.140625" style="16" customWidth="1"/>
@@ -2950,44 +2959,44 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>112</v>
+        <v>729</v>
       </c>
       <c r="B17" s="16" t="s">
-        <v>113</v>
+        <v>730</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>114</v>
+        <v>731</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>114</v>
+        <v>731</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="B18" s="16" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="B19" s="16" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
@@ -3001,7 +3010,7 @@
         <v>120</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>482</v>
+        <v>120</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
@@ -3014,246 +3023,246 @@
       <c r="C21" s="7" t="s">
         <v>120</v>
       </c>
-      <c r="D21" t="s">
-        <v>620</v>
+      <c r="D21" s="7" t="s">
+        <v>482</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="B22" s="16" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>123</v>
-      </c>
-      <c r="D22" s="7" t="s">
-        <v>123</v>
+        <v>120</v>
+      </c>
+      <c r="D22" t="s">
+        <v>620</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="B23" s="16" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="B24" s="16" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="B25" s="16" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="B26" s="16" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="B27" s="16" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="B28" s="16" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="D28" s="7" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="B29" s="16" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="B30" s="16" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="D30" s="7" t="s">
-        <v>478</v>
+        <v>144</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="B31" s="16" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="D31" s="7" t="s">
-        <v>150</v>
+        <v>478</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>314</v>
+        <v>148</v>
       </c>
       <c r="B32" s="16" t="s">
-        <v>110</v>
+        <v>149</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>111</v>
+        <v>150</v>
       </c>
       <c r="D32" s="7" t="s">
-        <v>479</v>
+        <v>150</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>151</v>
+        <v>314</v>
       </c>
       <c r="B33" s="16" t="s">
-        <v>152</v>
+        <v>110</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>153</v>
+        <v>111</v>
       </c>
       <c r="D33" s="7" t="s">
-        <v>153</v>
+        <v>479</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>124</v>
+        <v>151</v>
       </c>
       <c r="B34" s="16" t="s">
-        <v>125</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="D34" s="1" t="s">
-        <v>126</v>
+        <v>152</v>
+      </c>
+      <c r="C34" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="D34" s="7" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>154</v>
+        <v>124</v>
       </c>
       <c r="B35" s="16" t="s">
-        <v>155</v>
+        <v>125</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>156</v>
+        <v>126</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>156</v>
+        <v>126</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>315</v>
+        <v>154</v>
       </c>
       <c r="B36" s="16" t="s">
-        <v>146</v>
-      </c>
-      <c r="C36" s="7" t="s">
-        <v>147</v>
-      </c>
-      <c r="D36" s="7" t="s">
-        <v>480</v>
+        <v>155</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>154</v>
+        <v>315</v>
       </c>
       <c r="B37" s="16" t="s">
-        <v>155</v>
-      </c>
-      <c r="C37" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="D37" s="1" t="s">
-        <v>156</v>
+        <v>146</v>
+      </c>
+      <c r="C37" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="D37" s="7" t="s">
+        <v>480</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>163</v>
+        <v>154</v>
       </c>
       <c r="B38" s="16" t="s">
-        <v>164</v>
+        <v>155</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>165</v>
+        <v>156</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>165</v>
+        <v>156</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
@@ -3266,22 +3275,22 @@
       <c r="C39" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="D39" t="s">
-        <v>619</v>
+      <c r="D39" s="1" t="s">
+        <v>165</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="B40" s="16" t="s">
-        <v>158</v>
-      </c>
-      <c r="C40" s="7" t="s">
-        <v>159</v>
-      </c>
-      <c r="D40" s="7" t="s">
-        <v>159</v>
+        <v>164</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="D40" t="s">
+        <v>619</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
@@ -3295,329 +3304,329 @@
         <v>159</v>
       </c>
       <c r="D41" s="7" t="s">
-        <v>481</v>
+        <v>159</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
-        <v>112</v>
+        <v>157</v>
       </c>
       <c r="B42" s="16" t="s">
-        <v>113</v>
+        <v>158</v>
       </c>
       <c r="C42" s="7" t="s">
-        <v>114</v>
+        <v>159</v>
       </c>
       <c r="D42" s="7" t="s">
-        <v>114</v>
+        <v>481</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>160</v>
+        <v>112</v>
       </c>
       <c r="B43" s="16" t="s">
-        <v>161</v>
-      </c>
-      <c r="C43" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="D43" s="1" t="s">
-        <v>162</v>
+        <v>113</v>
+      </c>
+      <c r="C43" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="D43" s="7" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B44" s="16" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
-        <v>154</v>
+        <v>163</v>
       </c>
       <c r="B45" s="16" t="s">
-        <v>155</v>
+        <v>164</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>156</v>
+        <v>165</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>156</v>
+        <v>165</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="B46" s="18" t="s">
-        <v>353</v>
+        <v>154</v>
+      </c>
+      <c r="B46" s="16" t="s">
+        <v>155</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>167</v>
+        <v>156</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>167</v>
+        <v>156</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="B47" s="18" t="s">
+        <v>353</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="D47" s="1" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A48" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="B47" s="16" t="s">
+      <c r="B48" s="16" t="s">
         <v>169</v>
       </c>
-      <c r="C47" s="1" t="s">
+      <c r="C48" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="D47" s="1" t="s">
+      <c r="D48" s="1" t="s">
         <v>170</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" s="9" t="s">
-        <v>354</v>
-      </c>
-      <c r="B48" s="10" t="s">
-        <v>356</v>
-      </c>
-      <c r="C48" s="9" t="s">
-        <v>355</v>
-      </c>
-      <c r="D48" s="9" t="s">
-        <v>355</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="9" t="s">
-        <v>451</v>
+        <v>354</v>
       </c>
       <c r="B49" s="10" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="C49" s="9" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
       <c r="D49" s="9" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="9" t="s">
-        <v>361</v>
+        <v>451</v>
       </c>
       <c r="B50" s="10" t="s">
-        <v>363</v>
+        <v>359</v>
       </c>
       <c r="C50" s="9" t="s">
-        <v>362</v>
+        <v>358</v>
       </c>
       <c r="D50" s="9" t="s">
-        <v>362</v>
+        <v>358</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="9" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="B51" s="10" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="C51" s="9" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="D51" s="9" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="9" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B52" s="10" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="C52" s="9" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="D52" s="9" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" s="9" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="B53" s="10" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="C53" s="9" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="D53" s="9" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" s="9" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="B54" s="10" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
       <c r="C54" s="9" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="D54" s="9" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" s="9" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="B55" s="10" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
       <c r="C55" s="9" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="D55" s="9" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="9" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
       <c r="B56" s="10" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
       <c r="C56" s="9" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
       <c r="D56" s="9" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" s="9" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="B57" s="10" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
       <c r="C57" s="9" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
       <c r="D57" s="9" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" s="9" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="B58" s="10" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
       <c r="C58" s="9" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="D58" s="9" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" s="9" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
       <c r="B59" s="10" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="C59" s="9" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
       <c r="D59" s="9" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" s="9" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
       <c r="B60" s="10" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
       <c r="C60" s="9" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
       <c r="D60" s="9" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" s="9" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
       <c r="B61" s="10" t="s">
-        <v>396</v>
-      </c>
-      <c r="C61" s="1" t="s">
-        <v>395</v>
-      </c>
-      <c r="D61" s="1" t="s">
-        <v>395</v>
+        <v>393</v>
+      </c>
+      <c r="C61" s="9" t="s">
+        <v>392</v>
+      </c>
+      <c r="D61" s="9" t="s">
+        <v>392</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" s="9" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="B62" s="10" t="s">
-        <v>399</v>
-      </c>
-      <c r="C62" s="9" t="s">
-        <v>398</v>
-      </c>
-      <c r="D62" s="9" t="s">
-        <v>398</v>
+        <v>396</v>
+      </c>
+      <c r="C62" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="D62" s="1" t="s">
+        <v>395</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" s="9" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="B63" s="10" t="s">
-        <v>402</v>
+        <v>399</v>
       </c>
       <c r="C63" s="9" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
       <c r="D63" s="9" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="9" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="B64" s="10" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
       <c r="C64" s="9" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
       <c r="D64" s="9" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
@@ -3631,426 +3640,440 @@
         <v>404</v>
       </c>
       <c r="D65" s="9" t="s">
-        <v>517</v>
+        <v>404</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" s="9" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
       <c r="B66" s="10" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="C66" s="9" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="D66" s="9" t="s">
-        <v>407</v>
+        <v>517</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" s="9" t="s">
+        <v>406</v>
+      </c>
+      <c r="B67" s="10" t="s">
+        <v>408</v>
+      </c>
+      <c r="C67" s="9" t="s">
+        <v>407</v>
+      </c>
+      <c r="D67" s="9" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A68" s="9" t="s">
         <v>409</v>
       </c>
-      <c r="B67" s="10" t="s">
+      <c r="B68" s="10" t="s">
         <v>411</v>
       </c>
-      <c r="C67" s="9" t="s">
+      <c r="C68" s="9" t="s">
         <v>410</v>
       </c>
-      <c r="D67" s="9" t="s">
+      <c r="D68" s="9" t="s">
         <v>410</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A68" s="11" t="s">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A69" s="11" t="s">
         <v>412</v>
       </c>
-      <c r="B68" s="10" t="s">
+      <c r="B69" s="10" t="s">
         <v>414</v>
       </c>
-      <c r="C68" s="11" t="s">
+      <c r="C69" s="11" t="s">
         <v>413</v>
       </c>
-      <c r="D68" s="11" t="s">
+      <c r="D69" s="11" t="s">
         <v>413</v>
-      </c>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A69" s="9" t="s">
-        <v>415</v>
-      </c>
-      <c r="B69" s="10" t="s">
-        <v>417</v>
-      </c>
-      <c r="C69" s="9" t="s">
-        <v>416</v>
-      </c>
-      <c r="D69" s="9" t="s">
-        <v>416</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" s="9" t="s">
-        <v>418</v>
+        <v>415</v>
       </c>
       <c r="B70" s="10" t="s">
-        <v>420</v>
-      </c>
-      <c r="C70" s="1" t="s">
-        <v>419</v>
-      </c>
-      <c r="D70" s="1" t="s">
-        <v>419</v>
+        <v>417</v>
+      </c>
+      <c r="C70" s="9" t="s">
+        <v>416</v>
+      </c>
+      <c r="D70" s="9" t="s">
+        <v>416</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" s="9" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
       <c r="B71" s="10" t="s">
-        <v>423</v>
-      </c>
-      <c r="C71" s="9" t="s">
-        <v>422</v>
-      </c>
-      <c r="D71" s="9" t="s">
-        <v>422</v>
+        <v>420</v>
+      </c>
+      <c r="C71" s="1" t="s">
+        <v>419</v>
+      </c>
+      <c r="D71" s="1" t="s">
+        <v>419</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" s="9" t="s">
+        <v>421</v>
+      </c>
+      <c r="B72" s="10" t="s">
+        <v>423</v>
+      </c>
+      <c r="C72" s="9" t="s">
+        <v>422</v>
+      </c>
+      <c r="D72" s="9" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A73" s="9" t="s">
         <v>424</v>
       </c>
-      <c r="B72" s="10" t="s">
+      <c r="B73" s="10" t="s">
         <v>426</v>
       </c>
-      <c r="C72" s="9" t="s">
+      <c r="C73" s="9" t="s">
         <v>425</v>
       </c>
-      <c r="D72" s="9" t="s">
+      <c r="D73" s="9" t="s">
         <v>425</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A73" s="11" t="s">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A74" s="11" t="s">
         <v>427</v>
       </c>
-      <c r="B73" s="10" t="s">
+      <c r="B74" s="10" t="s">
         <v>429</v>
       </c>
-      <c r="C73" s="11" t="s">
+      <c r="C74" s="11" t="s">
         <v>428</v>
       </c>
-      <c r="D73" s="11" t="s">
+      <c r="D74" s="11" t="s">
         <v>428</v>
-      </c>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A74" s="9" t="s">
-        <v>430</v>
-      </c>
-      <c r="B74" s="10" t="s">
-        <v>432</v>
-      </c>
-      <c r="C74" s="9" t="s">
-        <v>431</v>
-      </c>
-      <c r="D74" s="9" t="s">
-        <v>431</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" s="9" t="s">
-        <v>433</v>
+        <v>430</v>
       </c>
       <c r="B75" s="10" t="s">
-        <v>435</v>
+        <v>432</v>
       </c>
       <c r="C75" s="9" t="s">
-        <v>434</v>
+        <v>431</v>
       </c>
       <c r="D75" s="9" t="s">
-        <v>434</v>
+        <v>431</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" s="9" t="s">
-        <v>436</v>
+        <v>433</v>
       </c>
       <c r="B76" s="10" t="s">
-        <v>438</v>
+        <v>435</v>
       </c>
       <c r="C76" s="9" t="s">
-        <v>437</v>
+        <v>434</v>
       </c>
       <c r="D76" s="9" t="s">
-        <v>437</v>
+        <v>434</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" s="9" t="s">
-        <v>439</v>
+        <v>436</v>
       </c>
       <c r="B77" s="10" t="s">
-        <v>441</v>
-      </c>
-      <c r="C77" s="1" t="s">
-        <v>440</v>
-      </c>
-      <c r="D77" s="1" t="s">
-        <v>440</v>
+        <v>438</v>
+      </c>
+      <c r="C77" s="9" t="s">
+        <v>437</v>
+      </c>
+      <c r="D77" s="9" t="s">
+        <v>437</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" s="9" t="s">
-        <v>442</v>
+        <v>439</v>
       </c>
       <c r="B78" s="10" t="s">
-        <v>444</v>
-      </c>
-      <c r="C78" s="9" t="s">
-        <v>443</v>
-      </c>
-      <c r="D78" s="9" t="s">
-        <v>443</v>
+        <v>441</v>
+      </c>
+      <c r="C78" s="1" t="s">
+        <v>440</v>
+      </c>
+      <c r="D78" s="1" t="s">
+        <v>440</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" s="9" t="s">
-        <v>445</v>
+        <v>442</v>
       </c>
       <c r="B79" s="10" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
       <c r="C79" s="9" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
       <c r="D79" s="9" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" s="9" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
       <c r="B80" s="10" t="s">
-        <v>450</v>
+        <v>447</v>
       </c>
       <c r="C80" s="9" t="s">
-        <v>449</v>
+        <v>446</v>
       </c>
       <c r="D80" s="9" t="s">
-        <v>449</v>
+        <v>446</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" s="9" t="s">
-        <v>655</v>
-      </c>
-      <c r="B81" s="16" t="s">
-        <v>654</v>
+        <v>448</v>
+      </c>
+      <c r="B81" s="10" t="s">
+        <v>450</v>
       </c>
       <c r="C81" s="9" t="s">
-        <v>653</v>
-      </c>
-      <c r="D81" t="s">
-        <v>653</v>
+        <v>449</v>
+      </c>
+      <c r="D81" s="9" t="s">
+        <v>449</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" s="9" t="s">
-        <v>658</v>
+        <v>655</v>
       </c>
       <c r="B82" s="16" t="s">
-        <v>657</v>
+        <v>654</v>
       </c>
       <c r="C82" s="9" t="s">
-        <v>656</v>
-      </c>
-      <c r="D82" s="9" t="s">
-        <v>656</v>
+        <v>653</v>
+      </c>
+      <c r="D82" t="s">
+        <v>653</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" s="9" t="s">
-        <v>661</v>
+        <v>658</v>
       </c>
       <c r="B83" s="16" t="s">
-        <v>660</v>
-      </c>
-      <c r="C83" t="s">
-        <v>659</v>
-      </c>
-      <c r="D83" t="s">
-        <v>659</v>
+        <v>657</v>
+      </c>
+      <c r="C83" s="9" t="s">
+        <v>656</v>
+      </c>
+      <c r="D83" s="9" t="s">
+        <v>656</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" s="9" t="s">
+        <v>661</v>
+      </c>
+      <c r="B84" s="16" t="s">
+        <v>660</v>
+      </c>
+      <c r="C84" t="s">
+        <v>659</v>
+      </c>
+      <c r="D84" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A85" s="9" t="s">
         <v>664</v>
       </c>
-      <c r="B84" s="16" t="s">
+      <c r="B85" s="16" t="s">
         <v>662</v>
       </c>
-      <c r="C84" s="9" t="s">
+      <c r="C85" s="9" t="s">
         <v>663</v>
       </c>
-      <c r="D84" s="9" t="s">
+      <c r="D85" s="9" t="s">
         <v>663</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A85" s="1" t="s">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A86" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="B85" s="16" t="s">
+      <c r="B86" s="16" t="s">
         <v>146</v>
       </c>
-      <c r="C85" s="7" t="s">
+      <c r="C86" s="7" t="s">
         <v>147</v>
       </c>
-      <c r="D85" s="7" t="s">
+      <c r="D86" s="7" t="s">
         <v>147</v>
-      </c>
-    </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A86" s="21" t="s">
-        <v>677</v>
-      </c>
-      <c r="B86" s="16" t="s">
-        <v>687</v>
-      </c>
-      <c r="C86" t="s">
-        <v>667</v>
-      </c>
-      <c r="D86" t="s">
-        <v>667</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" s="21" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="B87" s="16" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="C87" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="D87" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" s="21" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="B88" s="16" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="C88" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="D88" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" s="21" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="B89" s="16" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="C89" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="D89" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" s="21" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="B90" s="16" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="C90" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="D90" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" s="21" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="B91" s="16" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="C91" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="D91" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" s="21" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="B92" s="16" t="s">
-        <v>694</v>
+        <v>692</v>
       </c>
       <c r="C92" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="D92" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" s="21" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="B93" s="16" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="C93" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="D93" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" s="21" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="B94" s="16" t="s">
-        <v>695</v>
+        <v>693</v>
       </c>
       <c r="C94" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="D94" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" s="21" t="s">
+        <v>685</v>
+      </c>
+      <c r="B95" s="16" t="s">
+        <v>695</v>
+      </c>
+      <c r="C95" t="s">
+        <v>675</v>
+      </c>
+      <c r="D95" t="s">
+        <v>675</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A96" s="21" t="s">
         <v>686</v>
       </c>
-      <c r="B95" s="16" t="s">
+      <c r="B96" s="16" t="s">
         <v>696</v>
       </c>
-      <c r="C95" t="s">
+      <c r="C96" t="s">
         <v>676</v>
       </c>
-      <c r="D95" t="s">
+      <c r="D96" t="s">
         <v>676</v>
       </c>
     </row>

</xml_diff>